<commit_message>
add maps with spatial distribution of pollution
</commit_message>
<xml_diff>
--- a/02_Output/Descriptives/Table_Municipality_Summary_Contaminants_Estimators.xlsx
+++ b/02_Output/Descriptives/Table_Municipality_Summary_Contaminants_Estimators.xlsx
@@ -1,24 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/estela_blanco_uc_cl/Documents/ANID Iniciación_2024_2027/Contamination_PTB_G-Formula/02_Output/Descriptives/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_C5AEF11DC05F1BC0A2E45A52F37BD2720AC5D38A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E427DC7-F3DA-BB4D-93C0-9B80B259EED5}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="mun_summary_long" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">mun_summary_long!$A$1:$H$397</definedName>
-  </definedNames>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -3016,8 +3007,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3065,21 +3056,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3117,7 +3100,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -3151,7 +3134,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -3186,10 +3168,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3362,12 +3343,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H397"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3393,7 +3373,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>13101</v>
       </c>
@@ -3419,7 +3399,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>13101</v>
       </c>
@@ -3445,7 +3425,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>13101</v>
       </c>
@@ -3471,7 +3451,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>13101</v>
       </c>
@@ -3497,7 +3477,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>13101</v>
       </c>
@@ -3523,7 +3503,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>13101</v>
       </c>
@@ -3549,7 +3529,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>13101</v>
       </c>
@@ -3575,7 +3555,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8">
       <c r="A9">
         <v>13101</v>
       </c>
@@ -3601,7 +3581,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8">
       <c r="A10">
         <v>13101</v>
       </c>
@@ -3627,7 +3607,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8">
       <c r="A11">
         <v>13101</v>
       </c>
@@ -3653,7 +3633,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8">
       <c r="A12">
         <v>13101</v>
       </c>
@@ -3679,7 +3659,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8">
       <c r="A13">
         <v>13101</v>
       </c>
@@ -3705,7 +3685,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8">
       <c r="A14">
         <v>13102</v>
       </c>
@@ -3731,7 +3711,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8">
       <c r="A15">
         <v>13102</v>
       </c>
@@ -3757,7 +3737,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8">
       <c r="A16">
         <v>13102</v>
       </c>
@@ -3783,7 +3763,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8">
       <c r="A17">
         <v>13102</v>
       </c>
@@ -3809,7 +3789,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8">
       <c r="A18">
         <v>13102</v>
       </c>
@@ -3835,7 +3815,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8">
       <c r="A19">
         <v>13102</v>
       </c>
@@ -3861,7 +3841,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8">
       <c r="A20">
         <v>13102</v>
       </c>
@@ -3887,7 +3867,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8">
       <c r="A21">
         <v>13102</v>
       </c>
@@ -3913,7 +3893,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8">
       <c r="A22">
         <v>13102</v>
       </c>
@@ -3939,7 +3919,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8">
       <c r="A23">
         <v>13102</v>
       </c>
@@ -3965,7 +3945,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8">
       <c r="A24">
         <v>13102</v>
       </c>
@@ -3991,7 +3971,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8">
       <c r="A25">
         <v>13102</v>
       </c>
@@ -4017,7 +3997,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8">
       <c r="A26">
         <v>13103</v>
       </c>
@@ -4043,7 +4023,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8">
       <c r="A27">
         <v>13103</v>
       </c>
@@ -4069,7 +4049,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8">
       <c r="A28">
         <v>13103</v>
       </c>
@@ -4095,7 +4075,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8">
       <c r="A29">
         <v>13103</v>
       </c>
@@ -4121,7 +4101,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8">
       <c r="A30">
         <v>13103</v>
       </c>
@@ -4147,7 +4127,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8">
       <c r="A31">
         <v>13103</v>
       </c>
@@ -4173,7 +4153,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8">
       <c r="A32">
         <v>13103</v>
       </c>
@@ -4199,7 +4179,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8">
       <c r="A33">
         <v>13103</v>
       </c>
@@ -4225,7 +4205,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8">
       <c r="A34">
         <v>13103</v>
       </c>
@@ -4251,7 +4231,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8">
       <c r="A35">
         <v>13103</v>
       </c>
@@ -4277,7 +4257,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8">
       <c r="A36">
         <v>13103</v>
       </c>
@@ -4303,7 +4283,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8">
       <c r="A37">
         <v>13103</v>
       </c>
@@ -4329,7 +4309,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8">
       <c r="A38">
         <v>13104</v>
       </c>
@@ -4355,7 +4335,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8">
       <c r="A39">
         <v>13104</v>
       </c>
@@ -4381,7 +4361,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8">
       <c r="A40">
         <v>13104</v>
       </c>
@@ -4407,7 +4387,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8">
       <c r="A41">
         <v>13104</v>
       </c>
@@ -4433,7 +4413,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8">
       <c r="A42">
         <v>13104</v>
       </c>
@@ -4459,7 +4439,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8">
       <c r="A43">
         <v>13104</v>
       </c>
@@ -4485,7 +4465,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8">
       <c r="A44">
         <v>13104</v>
       </c>
@@ -4511,7 +4491,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8">
       <c r="A45">
         <v>13104</v>
       </c>
@@ -4537,7 +4517,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8">
       <c r="A46">
         <v>13104</v>
       </c>
@@ -4563,7 +4543,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8">
       <c r="A47">
         <v>13104</v>
       </c>
@@ -4589,7 +4569,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8">
       <c r="A48">
         <v>13104</v>
       </c>
@@ -4615,7 +4595,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8">
       <c r="A49">
         <v>13104</v>
       </c>
@@ -4641,7 +4621,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8">
       <c r="A50">
         <v>13105</v>
       </c>
@@ -4667,7 +4647,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8">
       <c r="A51">
         <v>13105</v>
       </c>
@@ -4693,7 +4673,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8">
       <c r="A52">
         <v>13105</v>
       </c>
@@ -4719,7 +4699,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8">
       <c r="A53">
         <v>13105</v>
       </c>
@@ -4745,7 +4725,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8">
       <c r="A54">
         <v>13105</v>
       </c>
@@ -4771,7 +4751,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8">
       <c r="A55">
         <v>13105</v>
       </c>
@@ -4797,7 +4777,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8">
       <c r="A56">
         <v>13105</v>
       </c>
@@ -4823,7 +4803,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8">
       <c r="A57">
         <v>13105</v>
       </c>
@@ -4849,7 +4829,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8">
       <c r="A58">
         <v>13105</v>
       </c>
@@ -4875,7 +4855,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8">
       <c r="A59">
         <v>13105</v>
       </c>
@@ -4901,7 +4881,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8">
       <c r="A60">
         <v>13105</v>
       </c>
@@ -4927,7 +4907,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8">
       <c r="A61">
         <v>13105</v>
       </c>
@@ -4953,7 +4933,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8">
       <c r="A62">
         <v>13106</v>
       </c>
@@ -4979,7 +4959,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8">
       <c r="A63">
         <v>13106</v>
       </c>
@@ -5005,7 +4985,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8">
       <c r="A64">
         <v>13106</v>
       </c>
@@ -5031,7 +5011,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8">
       <c r="A65">
         <v>13106</v>
       </c>
@@ -5057,7 +5037,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8">
       <c r="A66">
         <v>13106</v>
       </c>
@@ -5083,7 +5063,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8">
       <c r="A67">
         <v>13106</v>
       </c>
@@ -5109,7 +5089,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8">
       <c r="A68">
         <v>13106</v>
       </c>
@@ -5135,7 +5115,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8">
       <c r="A69">
         <v>13106</v>
       </c>
@@ -5161,7 +5141,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8">
       <c r="A70">
         <v>13106</v>
       </c>
@@ -5187,7 +5167,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8">
       <c r="A71">
         <v>13106</v>
       </c>
@@ -5213,7 +5193,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8">
       <c r="A72">
         <v>13106</v>
       </c>
@@ -5239,7 +5219,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8">
       <c r="A73">
         <v>13106</v>
       </c>
@@ -5265,7 +5245,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8">
       <c r="A74">
         <v>13107</v>
       </c>
@@ -5291,7 +5271,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8">
       <c r="A75">
         <v>13107</v>
       </c>
@@ -5317,7 +5297,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8">
       <c r="A76">
         <v>13107</v>
       </c>
@@ -5343,7 +5323,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8">
       <c r="A77">
         <v>13107</v>
       </c>
@@ -5369,7 +5349,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8">
       <c r="A78">
         <v>13107</v>
       </c>
@@ -5395,7 +5375,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8">
       <c r="A79">
         <v>13107</v>
       </c>
@@ -5421,7 +5401,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8">
       <c r="A80">
         <v>13107</v>
       </c>
@@ -5447,7 +5427,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8">
       <c r="A81">
         <v>13107</v>
       </c>
@@ -5473,7 +5453,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:8">
       <c r="A82">
         <v>13107</v>
       </c>
@@ -5499,7 +5479,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8">
       <c r="A83">
         <v>13107</v>
       </c>
@@ -5525,7 +5505,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:8">
       <c r="A84">
         <v>13107</v>
       </c>
@@ -5551,7 +5531,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:8">
       <c r="A85">
         <v>13107</v>
       </c>
@@ -5577,7 +5557,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8">
       <c r="A86">
         <v>13108</v>
       </c>
@@ -5603,7 +5583,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:8">
       <c r="A87">
         <v>13108</v>
       </c>
@@ -5629,7 +5609,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8">
       <c r="A88">
         <v>13108</v>
       </c>
@@ -5655,7 +5635,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8">
       <c r="A89">
         <v>13108</v>
       </c>
@@ -5681,7 +5661,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8">
       <c r="A90">
         <v>13108</v>
       </c>
@@ -5707,7 +5687,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8">
       <c r="A91">
         <v>13108</v>
       </c>
@@ -5733,7 +5713,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:8">
       <c r="A92">
         <v>13108</v>
       </c>
@@ -5759,7 +5739,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:8">
       <c r="A93">
         <v>13108</v>
       </c>
@@ -5785,7 +5765,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8">
       <c r="A94">
         <v>13108</v>
       </c>
@@ -5811,7 +5791,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:8">
       <c r="A95">
         <v>13108</v>
       </c>
@@ -5837,7 +5817,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:8">
       <c r="A96">
         <v>13108</v>
       </c>
@@ -5863,7 +5843,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8">
       <c r="A97">
         <v>13108</v>
       </c>
@@ -5889,7 +5869,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8">
       <c r="A98">
         <v>13109</v>
       </c>
@@ -5915,7 +5895,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8">
       <c r="A99">
         <v>13109</v>
       </c>
@@ -5941,7 +5921,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:8">
       <c r="A100">
         <v>13109</v>
       </c>
@@ -5967,7 +5947,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:8">
       <c r="A101">
         <v>13109</v>
       </c>
@@ -5993,7 +5973,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:8">
       <c r="A102">
         <v>13109</v>
       </c>
@@ -6019,7 +5999,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:8">
       <c r="A103">
         <v>13109</v>
       </c>
@@ -6045,7 +6025,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:8">
       <c r="A104">
         <v>13109</v>
       </c>
@@ -6071,7 +6051,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:8">
       <c r="A105">
         <v>13109</v>
       </c>
@@ -6097,7 +6077,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:8">
       <c r="A106">
         <v>13109</v>
       </c>
@@ -6123,7 +6103,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:8">
       <c r="A107">
         <v>13109</v>
       </c>
@@ -6149,7 +6129,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:8">
       <c r="A108">
         <v>13109</v>
       </c>
@@ -6175,7 +6155,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:8">
       <c r="A109">
         <v>13109</v>
       </c>
@@ -6201,7 +6181,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:8">
       <c r="A110">
         <v>13110</v>
       </c>
@@ -6227,7 +6207,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:8">
       <c r="A111">
         <v>13110</v>
       </c>
@@ -6253,7 +6233,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:8">
       <c r="A112">
         <v>13110</v>
       </c>
@@ -6279,7 +6259,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:8">
       <c r="A113">
         <v>13110</v>
       </c>
@@ -6305,7 +6285,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:8">
       <c r="A114">
         <v>13110</v>
       </c>
@@ -6331,7 +6311,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:8">
       <c r="A115">
         <v>13110</v>
       </c>
@@ -6357,7 +6337,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:8">
       <c r="A116">
         <v>13110</v>
       </c>
@@ -6383,7 +6363,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8">
       <c r="A117">
         <v>13110</v>
       </c>
@@ -6409,7 +6389,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:8">
       <c r="A118">
         <v>13110</v>
       </c>
@@ -6435,7 +6415,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:8">
       <c r="A119">
         <v>13110</v>
       </c>
@@ -6461,7 +6441,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:8">
       <c r="A120">
         <v>13110</v>
       </c>
@@ -6487,7 +6467,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:8">
       <c r="A121">
         <v>13110</v>
       </c>
@@ -6513,7 +6493,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:8">
       <c r="A122">
         <v>13111</v>
       </c>
@@ -6539,7 +6519,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:8">
       <c r="A123">
         <v>13111</v>
       </c>
@@ -6565,7 +6545,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:8">
       <c r="A124">
         <v>13111</v>
       </c>
@@ -6591,7 +6571,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:8">
       <c r="A125">
         <v>13111</v>
       </c>
@@ -6617,7 +6597,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:8">
       <c r="A126">
         <v>13111</v>
       </c>
@@ -6643,7 +6623,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:8">
       <c r="A127">
         <v>13111</v>
       </c>
@@ -6669,7 +6649,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:8">
       <c r="A128">
         <v>13111</v>
       </c>
@@ -6695,7 +6675,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:8">
       <c r="A129">
         <v>13111</v>
       </c>
@@ -6721,7 +6701,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:8">
       <c r="A130">
         <v>13111</v>
       </c>
@@ -6747,7 +6727,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:8">
       <c r="A131">
         <v>13111</v>
       </c>
@@ -6773,7 +6753,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:8">
       <c r="A132">
         <v>13111</v>
       </c>
@@ -6799,7 +6779,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:8">
       <c r="A133">
         <v>13111</v>
       </c>
@@ -6825,7 +6805,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:8">
       <c r="A134">
         <v>13112</v>
       </c>
@@ -6851,7 +6831,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:8">
       <c r="A135">
         <v>13112</v>
       </c>
@@ -6877,7 +6857,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:8">
       <c r="A136">
         <v>13112</v>
       </c>
@@ -6903,7 +6883,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:8">
       <c r="A137">
         <v>13112</v>
       </c>
@@ -6929,7 +6909,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:8">
       <c r="A138">
         <v>13112</v>
       </c>
@@ -6955,7 +6935,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:8">
       <c r="A139">
         <v>13112</v>
       </c>
@@ -6981,7 +6961,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:8">
       <c r="A140">
         <v>13112</v>
       </c>
@@ -7007,7 +6987,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:8">
       <c r="A141">
         <v>13112</v>
       </c>
@@ -7033,7 +7013,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:8">
       <c r="A142">
         <v>13112</v>
       </c>
@@ -7059,7 +7039,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:8">
       <c r="A143">
         <v>13112</v>
       </c>
@@ -7085,7 +7065,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:8">
       <c r="A144">
         <v>13112</v>
       </c>
@@ -7111,7 +7091,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:8">
       <c r="A145">
         <v>13112</v>
       </c>
@@ -7137,7 +7117,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:8">
       <c r="A146">
         <v>13113</v>
       </c>
@@ -7163,7 +7143,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:8">
       <c r="A147">
         <v>13113</v>
       </c>
@@ -7189,7 +7169,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:8">
       <c r="A148">
         <v>13113</v>
       </c>
@@ -7215,7 +7195,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:8">
       <c r="A149">
         <v>13113</v>
       </c>
@@ -7241,7 +7221,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:8">
       <c r="A150">
         <v>13113</v>
       </c>
@@ -7267,7 +7247,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:8">
       <c r="A151">
         <v>13113</v>
       </c>
@@ -7293,7 +7273,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:8">
       <c r="A152">
         <v>13113</v>
       </c>
@@ -7319,7 +7299,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:8">
       <c r="A153">
         <v>13113</v>
       </c>
@@ -7345,7 +7325,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:8">
       <c r="A154">
         <v>13113</v>
       </c>
@@ -7371,7 +7351,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:8">
       <c r="A155">
         <v>13113</v>
       </c>
@@ -7397,7 +7377,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:8">
       <c r="A156">
         <v>13113</v>
       </c>
@@ -7423,7 +7403,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:8">
       <c r="A157">
         <v>13113</v>
       </c>
@@ -7449,7 +7429,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:8">
       <c r="A158">
         <v>13114</v>
       </c>
@@ -7475,7 +7455,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:8">
       <c r="A159">
         <v>13114</v>
       </c>
@@ -7501,7 +7481,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:8">
       <c r="A160">
         <v>13114</v>
       </c>
@@ -7527,7 +7507,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:8">
       <c r="A161">
         <v>13114</v>
       </c>
@@ -7553,7 +7533,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:8">
       <c r="A162">
         <v>13114</v>
       </c>
@@ -7579,7 +7559,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:8">
       <c r="A163">
         <v>13114</v>
       </c>
@@ -7605,7 +7585,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:8">
       <c r="A164">
         <v>13114</v>
       </c>
@@ -7631,7 +7611,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:8">
       <c r="A165">
         <v>13114</v>
       </c>
@@ -7657,7 +7637,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:8">
       <c r="A166">
         <v>13114</v>
       </c>
@@ -7683,7 +7663,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:8">
       <c r="A167">
         <v>13114</v>
       </c>
@@ -7709,7 +7689,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:8">
       <c r="A168">
         <v>13114</v>
       </c>
@@ -7735,7 +7715,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:8">
       <c r="A169">
         <v>13114</v>
       </c>
@@ -7761,7 +7741,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:8">
       <c r="A170">
         <v>13115</v>
       </c>
@@ -7787,7 +7767,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:8">
       <c r="A171">
         <v>13115</v>
       </c>
@@ -7813,7 +7793,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:8">
       <c r="A172">
         <v>13115</v>
       </c>
@@ -7839,7 +7819,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:8">
       <c r="A173">
         <v>13115</v>
       </c>
@@ -7865,7 +7845,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:8">
       <c r="A174">
         <v>13115</v>
       </c>
@@ -7891,7 +7871,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:8">
       <c r="A175">
         <v>13115</v>
       </c>
@@ -7917,7 +7897,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:8">
       <c r="A176">
         <v>13115</v>
       </c>
@@ -7943,7 +7923,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:8">
       <c r="A177">
         <v>13115</v>
       </c>
@@ -7969,7 +7949,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:8">
       <c r="A178">
         <v>13115</v>
       </c>
@@ -7995,7 +7975,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:8">
       <c r="A179">
         <v>13115</v>
       </c>
@@ -8021,7 +8001,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:8">
       <c r="A180">
         <v>13115</v>
       </c>
@@ -8047,7 +8027,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:8">
       <c r="A181">
         <v>13115</v>
       </c>
@@ -8073,7 +8053,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:8">
       <c r="A182">
         <v>13116</v>
       </c>
@@ -8099,7 +8079,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:8">
       <c r="A183">
         <v>13116</v>
       </c>
@@ -8125,7 +8105,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:8">
       <c r="A184">
         <v>13116</v>
       </c>
@@ -8151,7 +8131,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:8">
       <c r="A185">
         <v>13116</v>
       </c>
@@ -8177,7 +8157,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:8">
       <c r="A186">
         <v>13116</v>
       </c>
@@ -8203,7 +8183,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:8">
       <c r="A187">
         <v>13116</v>
       </c>
@@ -8229,7 +8209,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:8">
       <c r="A188">
         <v>13116</v>
       </c>
@@ -8255,7 +8235,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:8">
       <c r="A189">
         <v>13116</v>
       </c>
@@ -8281,7 +8261,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:8">
       <c r="A190">
         <v>13116</v>
       </c>
@@ -8307,7 +8287,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:8">
       <c r="A191">
         <v>13116</v>
       </c>
@@ -8333,7 +8313,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:8">
       <c r="A192">
         <v>13116</v>
       </c>
@@ -8359,7 +8339,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:8">
       <c r="A193">
         <v>13116</v>
       </c>
@@ -8385,7 +8365,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:8">
       <c r="A194">
         <v>13117</v>
       </c>
@@ -8411,7 +8391,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:8">
       <c r="A195">
         <v>13117</v>
       </c>
@@ -8437,7 +8417,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:8">
       <c r="A196">
         <v>13117</v>
       </c>
@@ -8463,7 +8443,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:8">
       <c r="A197">
         <v>13117</v>
       </c>
@@ -8489,7 +8469,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:8">
       <c r="A198">
         <v>13117</v>
       </c>
@@ -8515,7 +8495,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:8">
       <c r="A199">
         <v>13117</v>
       </c>
@@ -8541,7 +8521,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:8">
       <c r="A200">
         <v>13117</v>
       </c>
@@ -8567,7 +8547,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:8">
       <c r="A201">
         <v>13117</v>
       </c>
@@ -8593,7 +8573,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:8">
       <c r="A202">
         <v>13117</v>
       </c>
@@ -8619,7 +8599,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:8">
       <c r="A203">
         <v>13117</v>
       </c>
@@ -8645,7 +8625,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:8">
       <c r="A204">
         <v>13117</v>
       </c>
@@ -8671,7 +8651,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:8">
       <c r="A205">
         <v>13117</v>
       </c>
@@ -8697,7 +8677,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:8">
       <c r="A206">
         <v>13118</v>
       </c>
@@ -8723,7 +8703,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:8">
       <c r="A207">
         <v>13118</v>
       </c>
@@ -8749,7 +8729,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:8">
       <c r="A208">
         <v>13118</v>
       </c>
@@ -8775,7 +8755,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:8">
       <c r="A209">
         <v>13118</v>
       </c>
@@ -8801,7 +8781,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:8">
       <c r="A210">
         <v>13118</v>
       </c>
@@ -8827,7 +8807,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:8">
       <c r="A211">
         <v>13118</v>
       </c>
@@ -8853,7 +8833,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:8">
       <c r="A212">
         <v>13118</v>
       </c>
@@ -8879,7 +8859,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:8">
       <c r="A213">
         <v>13118</v>
       </c>
@@ -8905,7 +8885,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:8">
       <c r="A214">
         <v>13118</v>
       </c>
@@ -8931,7 +8911,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:8">
       <c r="A215">
         <v>13118</v>
       </c>
@@ -8957,7 +8937,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:8">
       <c r="A216">
         <v>13118</v>
       </c>
@@ -8983,7 +8963,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:8">
       <c r="A217">
         <v>13118</v>
       </c>
@@ -9009,7 +8989,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:8">
       <c r="A218">
         <v>13119</v>
       </c>
@@ -9035,7 +9015,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:8">
       <c r="A219">
         <v>13119</v>
       </c>
@@ -9061,7 +9041,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:8">
       <c r="A220">
         <v>13119</v>
       </c>
@@ -9087,7 +9067,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:8">
       <c r="A221">
         <v>13119</v>
       </c>
@@ -9113,7 +9093,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:8">
       <c r="A222">
         <v>13119</v>
       </c>
@@ -9139,7 +9119,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:8">
       <c r="A223">
         <v>13119</v>
       </c>
@@ -9165,7 +9145,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:8">
       <c r="A224">
         <v>13119</v>
       </c>
@@ -9191,7 +9171,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:8">
       <c r="A225">
         <v>13119</v>
       </c>
@@ -9217,7 +9197,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:8">
       <c r="A226">
         <v>13119</v>
       </c>
@@ -9243,7 +9223,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:8">
       <c r="A227">
         <v>13119</v>
       </c>
@@ -9269,7 +9249,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:8">
       <c r="A228">
         <v>13119</v>
       </c>
@@ -9295,7 +9275,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="229" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:8">
       <c r="A229">
         <v>13119</v>
       </c>
@@ -9321,7 +9301,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="230" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:8">
       <c r="A230">
         <v>13120</v>
       </c>
@@ -9347,7 +9327,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="231" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:8">
       <c r="A231">
         <v>13120</v>
       </c>
@@ -9373,7 +9353,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:8">
       <c r="A232">
         <v>13120</v>
       </c>
@@ -9399,7 +9379,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:8">
       <c r="A233">
         <v>13120</v>
       </c>
@@ -9425,7 +9405,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="234" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:8">
       <c r="A234">
         <v>13120</v>
       </c>
@@ -9451,7 +9431,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="235" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:8">
       <c r="A235">
         <v>13120</v>
       </c>
@@ -9477,7 +9457,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="236" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:8">
       <c r="A236">
         <v>13120</v>
       </c>
@@ -9503,7 +9483,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="237" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:8">
       <c r="A237">
         <v>13120</v>
       </c>
@@ -9529,7 +9509,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="238" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:8">
       <c r="A238">
         <v>13120</v>
       </c>
@@ -9555,7 +9535,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="239" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:8">
       <c r="A239">
         <v>13120</v>
       </c>
@@ -9581,7 +9561,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="240" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:8">
       <c r="A240">
         <v>13120</v>
       </c>
@@ -9607,7 +9587,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="241" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:8">
       <c r="A241">
         <v>13120</v>
       </c>
@@ -9633,7 +9613,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="242" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:8">
       <c r="A242">
         <v>13121</v>
       </c>
@@ -9659,7 +9639,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="243" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:8">
       <c r="A243">
         <v>13121</v>
       </c>
@@ -9685,7 +9665,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:8">
       <c r="A244">
         <v>13121</v>
       </c>
@@ -9711,7 +9691,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="245" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:8">
       <c r="A245">
         <v>13121</v>
       </c>
@@ -9737,7 +9717,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="246" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:8">
       <c r="A246">
         <v>13121</v>
       </c>
@@ -9763,7 +9743,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="247" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:8">
       <c r="A247">
         <v>13121</v>
       </c>
@@ -9789,7 +9769,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="248" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:8">
       <c r="A248">
         <v>13121</v>
       </c>
@@ -9815,7 +9795,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="249" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:8">
       <c r="A249">
         <v>13121</v>
       </c>
@@ -9841,7 +9821,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="250" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:8">
       <c r="A250">
         <v>13121</v>
       </c>
@@ -9867,7 +9847,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="251" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:8">
       <c r="A251">
         <v>13121</v>
       </c>
@@ -9893,7 +9873,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="252" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:8">
       <c r="A252">
         <v>13121</v>
       </c>
@@ -9919,7 +9899,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="253" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:8">
       <c r="A253">
         <v>13121</v>
       </c>
@@ -9945,7 +9925,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="254" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:8">
       <c r="A254">
         <v>13122</v>
       </c>
@@ -9971,7 +9951,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="255" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:8">
       <c r="A255">
         <v>13122</v>
       </c>
@@ -9997,7 +9977,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="256" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:8">
       <c r="A256">
         <v>13122</v>
       </c>
@@ -10023,7 +10003,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:8">
       <c r="A257">
         <v>13122</v>
       </c>
@@ -10049,7 +10029,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="258" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:8">
       <c r="A258">
         <v>13122</v>
       </c>
@@ -10075,7 +10055,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="259" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:8">
       <c r="A259">
         <v>13122</v>
       </c>
@@ -10101,7 +10081,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="260" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:8">
       <c r="A260">
         <v>13122</v>
       </c>
@@ -10127,7 +10107,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="261" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:8">
       <c r="A261">
         <v>13122</v>
       </c>
@@ -10153,7 +10133,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="262" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:8">
       <c r="A262">
         <v>13122</v>
       </c>
@@ -10179,7 +10159,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="263" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:8">
       <c r="A263">
         <v>13122</v>
       </c>
@@ -10205,7 +10185,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="264" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:8">
       <c r="A264">
         <v>13122</v>
       </c>
@@ -10231,7 +10211,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="265" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:8">
       <c r="A265">
         <v>13122</v>
       </c>
@@ -10257,7 +10237,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="266" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:8">
       <c r="A266">
         <v>13123</v>
       </c>
@@ -10283,7 +10263,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="267" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:8">
       <c r="A267">
         <v>13123</v>
       </c>
@@ -10309,7 +10289,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="268" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:8">
       <c r="A268">
         <v>13123</v>
       </c>
@@ -10335,7 +10315,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="269" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:8">
       <c r="A269">
         <v>13123</v>
       </c>
@@ -10361,7 +10341,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="270" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:8">
       <c r="A270">
         <v>13123</v>
       </c>
@@ -10387,7 +10367,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="271" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:8">
       <c r="A271">
         <v>13123</v>
       </c>
@@ -10413,7 +10393,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="272" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:8">
       <c r="A272">
         <v>13123</v>
       </c>
@@ -10439,7 +10419,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="273" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:8">
       <c r="A273">
         <v>13123</v>
       </c>
@@ -10465,7 +10445,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="274" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:8">
       <c r="A274">
         <v>13123</v>
       </c>
@@ -10491,7 +10471,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="275" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:8">
       <c r="A275">
         <v>13123</v>
       </c>
@@ -10517,7 +10497,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="276" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:8">
       <c r="A276">
         <v>13123</v>
       </c>
@@ -10543,7 +10523,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="277" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:8">
       <c r="A277">
         <v>13123</v>
       </c>
@@ -10569,7 +10549,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="278" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:8">
       <c r="A278">
         <v>13124</v>
       </c>
@@ -10595,7 +10575,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="279" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:8">
       <c r="A279">
         <v>13124</v>
       </c>
@@ -10621,7 +10601,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="280" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:8">
       <c r="A280">
         <v>13124</v>
       </c>
@@ -10647,7 +10627,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="281" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:8">
       <c r="A281">
         <v>13124</v>
       </c>
@@ -10673,7 +10653,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="282" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:8">
       <c r="A282">
         <v>13124</v>
       </c>
@@ -10699,7 +10679,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="283" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:8">
       <c r="A283">
         <v>13124</v>
       </c>
@@ -10725,7 +10705,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="284" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:8">
       <c r="A284">
         <v>13124</v>
       </c>
@@ -10751,7 +10731,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="285" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:8">
       <c r="A285">
         <v>13124</v>
       </c>
@@ -10777,7 +10757,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="286" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:8">
       <c r="A286">
         <v>13124</v>
       </c>
@@ -10803,7 +10783,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="287" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:8">
       <c r="A287">
         <v>13124</v>
       </c>
@@ -10829,7 +10809,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="288" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:8">
       <c r="A288">
         <v>13124</v>
       </c>
@@ -10855,7 +10835,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="289" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:8">
       <c r="A289">
         <v>13124</v>
       </c>
@@ -10881,7 +10861,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="290" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:8">
       <c r="A290">
         <v>13125</v>
       </c>
@@ -10907,7 +10887,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="291" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:8">
       <c r="A291">
         <v>13125</v>
       </c>
@@ -10933,7 +10913,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="292" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:8">
       <c r="A292">
         <v>13125</v>
       </c>
@@ -10959,7 +10939,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:8">
       <c r="A293">
         <v>13125</v>
       </c>
@@ -10985,7 +10965,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="294" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:8">
       <c r="A294">
         <v>13125</v>
       </c>
@@ -11011,7 +10991,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="295" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:8">
       <c r="A295">
         <v>13125</v>
       </c>
@@ -11037,7 +11017,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="296" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:8">
       <c r="A296">
         <v>13125</v>
       </c>
@@ -11063,7 +11043,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="297" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:8">
       <c r="A297">
         <v>13125</v>
       </c>
@@ -11089,7 +11069,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="298" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:8">
       <c r="A298">
         <v>13125</v>
       </c>
@@ -11115,7 +11095,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="299" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:8">
       <c r="A299">
         <v>13125</v>
       </c>
@@ -11141,7 +11121,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="300" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:8">
       <c r="A300">
         <v>13125</v>
       </c>
@@ -11167,7 +11147,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="301" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:8">
       <c r="A301">
         <v>13125</v>
       </c>
@@ -11193,7 +11173,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="302" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:8">
       <c r="A302">
         <v>13126</v>
       </c>
@@ -11219,7 +11199,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="303" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:8">
       <c r="A303">
         <v>13126</v>
       </c>
@@ -11245,7 +11225,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="304" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:8">
       <c r="A304">
         <v>13126</v>
       </c>
@@ -11271,7 +11251,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="305" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:8">
       <c r="A305">
         <v>13126</v>
       </c>
@@ -11297,7 +11277,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="306" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:8">
       <c r="A306">
         <v>13126</v>
       </c>
@@ -11323,7 +11303,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="307" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:8">
       <c r="A307">
         <v>13126</v>
       </c>
@@ -11349,7 +11329,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="308" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:8">
       <c r="A308">
         <v>13126</v>
       </c>
@@ -11375,7 +11355,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="309" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:8">
       <c r="A309">
         <v>13126</v>
       </c>
@@ -11401,7 +11381,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="310" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:8">
       <c r="A310">
         <v>13126</v>
       </c>
@@ -11427,7 +11407,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="311" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:8">
       <c r="A311">
         <v>13126</v>
       </c>
@@ -11453,7 +11433,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="312" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:8">
       <c r="A312">
         <v>13126</v>
       </c>
@@ -11479,7 +11459,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="313" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:8">
       <c r="A313">
         <v>13126</v>
       </c>
@@ -11505,7 +11485,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="314" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:8">
       <c r="A314">
         <v>13127</v>
       </c>
@@ -11531,7 +11511,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="315" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:8">
       <c r="A315">
         <v>13127</v>
       </c>
@@ -11557,7 +11537,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="316" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:8">
       <c r="A316">
         <v>13127</v>
       </c>
@@ -11583,7 +11563,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="317" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:8">
       <c r="A317">
         <v>13127</v>
       </c>
@@ -11609,7 +11589,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="318" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:8">
       <c r="A318">
         <v>13127</v>
       </c>
@@ -11635,7 +11615,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="319" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:8">
       <c r="A319">
         <v>13127</v>
       </c>
@@ -11661,7 +11641,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="320" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:8">
       <c r="A320">
         <v>13127</v>
       </c>
@@ -11687,7 +11667,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="321" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:8">
       <c r="A321">
         <v>13127</v>
       </c>
@@ -11713,7 +11693,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="322" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:8">
       <c r="A322">
         <v>13127</v>
       </c>
@@ -11739,7 +11719,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="323" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:8">
       <c r="A323">
         <v>13127</v>
       </c>
@@ -11765,7 +11745,7 @@
         <v>838</v>
       </c>
     </row>
-    <row r="324" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:8">
       <c r="A324">
         <v>13127</v>
       </c>
@@ -11791,7 +11771,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="325" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:8">
       <c r="A325">
         <v>13127</v>
       </c>
@@ -11817,7 +11797,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="326" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:8">
       <c r="A326">
         <v>13128</v>
       </c>
@@ -11843,7 +11823,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="327" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:8">
       <c r="A327">
         <v>13128</v>
       </c>
@@ -11869,7 +11849,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="328" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:8">
       <c r="A328">
         <v>13128</v>
       </c>
@@ -11895,7 +11875,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="329" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:8">
       <c r="A329">
         <v>13128</v>
       </c>
@@ -11921,7 +11901,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="330" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:8">
       <c r="A330">
         <v>13128</v>
       </c>
@@ -11947,7 +11927,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="331" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:8">
       <c r="A331">
         <v>13128</v>
       </c>
@@ -11973,7 +11953,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="332" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:8">
       <c r="A332">
         <v>13128</v>
       </c>
@@ -11999,7 +11979,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="333" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:8">
       <c r="A333">
         <v>13128</v>
       </c>
@@ -12025,7 +12005,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="334" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:8">
       <c r="A334">
         <v>13128</v>
       </c>
@@ -12051,7 +12031,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="335" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:8">
       <c r="A335">
         <v>13128</v>
       </c>
@@ -12077,7 +12057,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="336" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:8">
       <c r="A336">
         <v>13128</v>
       </c>
@@ -12103,7 +12083,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="337" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:8">
       <c r="A337">
         <v>13128</v>
       </c>
@@ -12129,7 +12109,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="338" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:8">
       <c r="A338">
         <v>13129</v>
       </c>
@@ -12155,7 +12135,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="339" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:8">
       <c r="A339">
         <v>13129</v>
       </c>
@@ -12181,7 +12161,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="340" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:8">
       <c r="A340">
         <v>13129</v>
       </c>
@@ -12207,7 +12187,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="341" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:8">
       <c r="A341">
         <v>13129</v>
       </c>
@@ -12233,7 +12213,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="342" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:8">
       <c r="A342">
         <v>13129</v>
       </c>
@@ -12259,7 +12239,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="343" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:8">
       <c r="A343">
         <v>13129</v>
       </c>
@@ -12285,7 +12265,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="344" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:8">
       <c r="A344">
         <v>13129</v>
       </c>
@@ -12311,7 +12291,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="345" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:8">
       <c r="A345">
         <v>13129</v>
       </c>
@@ -12337,7 +12317,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="346" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:8">
       <c r="A346">
         <v>13129</v>
       </c>
@@ -12363,7 +12343,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="347" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:8">
       <c r="A347">
         <v>13129</v>
       </c>
@@ -12389,7 +12369,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="348" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:8">
       <c r="A348">
         <v>13129</v>
       </c>
@@ -12415,7 +12395,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="349" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:8">
       <c r="A349">
         <v>13129</v>
       </c>
@@ -12441,7 +12421,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="350" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:8">
       <c r="A350">
         <v>13130</v>
       </c>
@@ -12467,7 +12447,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="351" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:8">
       <c r="A351">
         <v>13130</v>
       </c>
@@ -12493,7 +12473,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="352" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:8">
       <c r="A352">
         <v>13130</v>
       </c>
@@ -12519,7 +12499,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="353" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:8">
       <c r="A353">
         <v>13130</v>
       </c>
@@ -12545,7 +12525,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="354" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:8">
       <c r="A354">
         <v>13130</v>
       </c>
@@ -12571,7 +12551,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="355" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:8">
       <c r="A355">
         <v>13130</v>
       </c>
@@ -12597,7 +12577,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="356" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:8">
       <c r="A356">
         <v>13130</v>
       </c>
@@ -12623,7 +12603,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="357" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:8">
       <c r="A357">
         <v>13130</v>
       </c>
@@ -12649,7 +12629,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="358" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:8">
       <c r="A358">
         <v>13130</v>
       </c>
@@ -12675,7 +12655,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="359" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="359" spans="1:8">
       <c r="A359">
         <v>13130</v>
       </c>
@@ -12701,7 +12681,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="360" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="360" spans="1:8">
       <c r="A360">
         <v>13130</v>
       </c>
@@ -12727,7 +12707,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="361" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:8">
       <c r="A361">
         <v>13130</v>
       </c>
@@ -12753,7 +12733,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="362" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="362" spans="1:8">
       <c r="A362">
         <v>13131</v>
       </c>
@@ -12779,7 +12759,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="363" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="363" spans="1:8">
       <c r="A363">
         <v>13131</v>
       </c>
@@ -12805,7 +12785,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="364" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:8">
       <c r="A364">
         <v>13131</v>
       </c>
@@ -12831,7 +12811,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="365" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:8">
       <c r="A365">
         <v>13131</v>
       </c>
@@ -12857,7 +12837,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="366" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:8">
       <c r="A366">
         <v>13131</v>
       </c>
@@ -12883,7 +12863,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="367" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:8">
       <c r="A367">
         <v>13131</v>
       </c>
@@ -12909,7 +12889,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="368" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:8">
       <c r="A368">
         <v>13131</v>
       </c>
@@ -12935,7 +12915,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="369" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:8">
       <c r="A369">
         <v>13131</v>
       </c>
@@ -12961,7 +12941,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="370" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="370" spans="1:8">
       <c r="A370">
         <v>13131</v>
       </c>
@@ -12987,7 +12967,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="371" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:8">
       <c r="A371">
         <v>13131</v>
       </c>
@@ -13013,7 +12993,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="372" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:8">
       <c r="A372">
         <v>13131</v>
       </c>
@@ -13039,7 +13019,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="373" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="373" spans="1:8">
       <c r="A373">
         <v>13131</v>
       </c>
@@ -13065,7 +13045,7 @@
         <v>940</v>
       </c>
     </row>
-    <row r="374" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:8">
       <c r="A374">
         <v>13132</v>
       </c>
@@ -13091,7 +13071,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="375" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:8">
       <c r="A375">
         <v>13132</v>
       </c>
@@ -13117,7 +13097,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="376" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="376" spans="1:8">
       <c r="A376">
         <v>13132</v>
       </c>
@@ -13143,7 +13123,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="377" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="377" spans="1:8">
       <c r="A377">
         <v>13132</v>
       </c>
@@ -13169,7 +13149,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="378" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="378" spans="1:8">
       <c r="A378">
         <v>13132</v>
       </c>
@@ -13195,7 +13175,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="379" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="379" spans="1:8">
       <c r="A379">
         <v>13132</v>
       </c>
@@ -13221,7 +13201,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="380" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="380" spans="1:8">
       <c r="A380">
         <v>13132</v>
       </c>
@@ -13247,7 +13227,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="381" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="381" spans="1:8">
       <c r="A381">
         <v>13132</v>
       </c>
@@ -13273,7 +13253,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="382" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="382" spans="1:8">
       <c r="A382">
         <v>13132</v>
       </c>
@@ -13299,7 +13279,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="383" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="383" spans="1:8">
       <c r="A383">
         <v>13132</v>
       </c>
@@ -13325,7 +13305,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="384" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="384" spans="1:8">
       <c r="A384">
         <v>13132</v>
       </c>
@@ -13351,7 +13331,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="385" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="385" spans="1:8">
       <c r="A385">
         <v>13132</v>
       </c>
@@ -13377,7 +13357,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="386" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="386" spans="1:8">
       <c r="A386">
         <v>13201</v>
       </c>
@@ -13403,7 +13383,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="387" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="387" spans="1:8">
       <c r="A387">
         <v>13201</v>
       </c>
@@ -13429,7 +13409,7 @@
         <v>974</v>
       </c>
     </row>
-    <row r="388" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="388" spans="1:8">
       <c r="A388">
         <v>13201</v>
       </c>
@@ -13455,7 +13435,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="389" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="389" spans="1:8">
       <c r="A389">
         <v>13201</v>
       </c>
@@ -13481,7 +13461,7 @@
         <v>979</v>
       </c>
     </row>
-    <row r="390" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="390" spans="1:8">
       <c r="A390">
         <v>13201</v>
       </c>
@@ -13507,7 +13487,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="391" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="391" spans="1:8">
       <c r="A391">
         <v>13201</v>
       </c>
@@ -13533,7 +13513,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="392" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="392" spans="1:8">
       <c r="A392">
         <v>13201</v>
       </c>
@@ -13559,7 +13539,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="393" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="393" spans="1:8">
       <c r="A393">
         <v>13201</v>
       </c>
@@ -13585,7 +13565,7 @@
         <v>987</v>
       </c>
     </row>
-    <row r="394" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="394" spans="1:8">
       <c r="A394">
         <v>13201</v>
       </c>
@@ -13611,7 +13591,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="395" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="395" spans="1:8">
       <c r="A395">
         <v>13201</v>
       </c>
@@ -13637,7 +13617,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="396" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="396" spans="1:8">
       <c r="A396">
         <v>13201</v>
       </c>
@@ -13663,7 +13643,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="397" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="397" spans="1:8">
       <c r="A397">
         <v>13201</v>
       </c>
@@ -13690,18 +13670,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H397" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Summer"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="3">
-      <filters>
-        <filter val="O3"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>